<commit_message>
Puliza file mapping Excel
</commit_message>
<xml_diff>
--- a/programma_lezioni_inglese_no_audio.xlsx
+++ b/programma_lezioni_inglese_no_audio.xlsx
@@ -1,25 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programma Lezioni" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modello Dati" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Logica Didattica" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Percorso MVP" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grammatica" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vocabolario" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comunicazione" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liste" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Struttura_Lezione" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Struttura_Quiz" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="struttura_quiz_guidato" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="struttura_quiz_finale" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Programma Lezioni" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Percorso MVP" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Grammatica" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Vocabolario" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Comunicazione" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Liste" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -758,23 +751,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TabRoadmap" displayName="TabRoadmap" ref="A4:H9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A4:H9"/>
-  <tableColumns count="8">
-    <tableColumn id="1" name="Fase"/>
-    <tableColumn id="2" name="Obiettivo"/>
-    <tableColumn id="3" name="Lezioni da Sviluppare"/>
-    <tableColumn id="4" name="Categorie Coinvolte"/>
-    <tableColumn id="5" name="Funzionalità Necessarie"/>
-    <tableColumn id="6" name="Priorità"/>
-    <tableColumn id="7" name="Complessità"/>
-    <tableColumn id="8" name="Dipendenze"/>
-  </tableColumns>
-</table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TabLezioniGRA" displayName="TabLezioniGRA" ref="A16:G73" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TabLezioniGRA" displayName="TabLezioniGRA" ref="A16:G73" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A16:G73"/>
   <tableColumns count="7">
     <tableColumn id="1" name="ID Lezione"/>
@@ -788,8 +765,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="TabStrutturaGRA" displayName="TabStrutturaGRA" ref="A4:E13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TabStrutturaGRA" displayName="TabStrutturaGRA" ref="A4:E13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:E13"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Ordine"/>
@@ -801,8 +778,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TabLezioniVOC" displayName="TabLezioniVOC" ref="A14:G31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="TabLezioniVOC" displayName="TabLezioniVOC" ref="A14:G31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A14:G31"/>
   <tableColumns count="7">
     <tableColumn id="1" name="ID Lezione"/>
@@ -816,8 +793,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TabStrutturaVOC" displayName="TabStrutturaVOC" ref="A4:E11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TabStrutturaVOC" displayName="TabStrutturaVOC" ref="A4:E11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:E11"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Ordine"/>
@@ -829,8 +806,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="TabLezioniCOM" displayName="TabLezioniCOM" ref="A15:G39" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="TabLezioniCOM" displayName="TabLezioniCOM" ref="A15:G39" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A15:G39"/>
   <tableColumns count="7">
     <tableColumn id="1" name="ID Lezione"/>
@@ -844,8 +821,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="TabStrutturaCOM" displayName="TabStrutturaCOM" ref="A4:E12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="TabStrutturaCOM" displayName="TabStrutturaCOM" ref="A4:E12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:E12"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Ordine"/>
@@ -9408,1330 +9385,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" style="40" min="1" max="1"/>
-    <col width="22" customWidth="1" style="40" min="2" max="2"/>
-    <col width="14" customWidth="1" style="40" min="3" max="3"/>
-    <col width="68" customWidth="1" style="40" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="81" t="inlineStr">
-        <is>
-          <t>STRUTTURA_LEZIONE — sezioni che compongono una lezione</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1" s="40">
-      <c r="A2" s="82" t="inlineStr">
-        <is>
-          <t>Tabella Neon: struttura_lezione (ex learning_sezionelezione). Una riga per sezione, ordinata da «ordine» (UNIQUE con lezione_id). I template per area sono nei fogli Grammatica / Vocabolario / Comunicazione.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="83" t="inlineStr">
-        <is>
-          <t>Colonna</t>
-        </is>
-      </c>
-      <c r="B4" s="83" t="inlineStr">
-        <is>
-          <t>Tipo Neon</t>
-        </is>
-      </c>
-      <c r="C4" s="83" t="inlineStr">
-        <is>
-          <t>Obbligatoria</t>
-        </is>
-      </c>
-      <c r="D4" s="83" t="inlineStr">
-        <is>
-          <t>Descrizione</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="84" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B5" s="84" t="inlineStr">
-        <is>
-          <t>bigint (identity)</t>
-        </is>
-      </c>
-      <c r="C5" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D5" s="84" t="inlineStr">
-        <is>
-          <t>Chiave primaria tecnica.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="84" t="inlineStr">
-        <is>
-          <t>lezione_id</t>
-        </is>
-      </c>
-      <c r="B6" s="84" t="inlineStr">
-        <is>
-          <t>varchar(32) FK</t>
-        </is>
-      </c>
-      <c r="C6" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D6" s="84" t="inlineStr">
-        <is>
-          <t>Riferimento a learning_lezione.id.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="84" t="inlineStr">
-        <is>
-          <t>ordine</t>
-        </is>
-      </c>
-      <c r="B7" s="84" t="inlineStr">
-        <is>
-          <t>smallint</t>
-        </is>
-      </c>
-      <c r="C7" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D7" s="84" t="inlineStr">
-        <is>
-          <t>Posizione della sezione. UNIQUE con lezione_id.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="84" t="inlineStr">
-        <is>
-          <t>tipo_sezione</t>
-        </is>
-      </c>
-      <c r="B8" s="84" t="inlineStr">
-        <is>
-          <t>varchar(80)</t>
-        </is>
-      </c>
-      <c r="C8" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D8" s="84" t="inlineStr">
-        <is>
-          <t>Nome della sezione, es. «Regola e uso».</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="84" t="inlineStr">
-        <is>
-          <t>contenuto</t>
-        </is>
-      </c>
-      <c r="B9" s="84" t="inlineStr">
-        <is>
-          <t>jsonb</t>
-        </is>
-      </c>
-      <c r="C9" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D9" s="84" t="inlineStr">
-        <is>
-          <t>Chiavi tipiche: titolo, testo, elementi. Con formato_web = todo contiene il segnaposto TODO_FONTE.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="84" t="inlineStr">
-        <is>
-          <t>formato_web</t>
-        </is>
-      </c>
-      <c r="B10" s="84" t="inlineStr">
-        <is>
-          <t>varchar(40)</t>
-        </is>
-      </c>
-      <c r="C10" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D10" s="84" t="inlineStr">
-        <is>
-          <t>Resa nel frontend: testo, lista, errore_box, todo.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" style="40" min="1" max="1"/>
-    <col width="22" customWidth="1" style="40" min="2" max="2"/>
-    <col width="14" customWidth="1" style="40" min="3" max="3"/>
-    <col width="68" customWidth="1" style="40" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="81" t="inlineStr">
-        <is>
-          <t>STRUTTURA_QUIZ — parte esercitativa della lezione</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1" s="40">
-      <c r="A2" s="82" t="inlineStr">
-        <is>
-          <t>Tabella Neon: struttura_quiz (ex learning_quiz). Al massimo due righe per lezione, una per modalita. I quesiti stanno nei fogli struttura_quiz_guidato e struttura_quiz_finale.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="83" t="inlineStr">
-        <is>
-          <t>Colonna</t>
-        </is>
-      </c>
-      <c r="B4" s="83" t="inlineStr">
-        <is>
-          <t>Tipo Neon</t>
-        </is>
-      </c>
-      <c r="C4" s="83" t="inlineStr">
-        <is>
-          <t>Obbligatoria</t>
-        </is>
-      </c>
-      <c r="D4" s="83" t="inlineStr">
-        <is>
-          <t>Descrizione</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="84" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B5" s="84" t="inlineStr">
-        <is>
-          <t>bigint (identity)</t>
-        </is>
-      </c>
-      <c r="C5" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D5" s="84" t="inlineStr">
-        <is>
-          <t>Chiave primaria tecnica.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="84" t="inlineStr">
-        <is>
-          <t>lezione_id</t>
-        </is>
-      </c>
-      <c r="B6" s="84" t="inlineStr">
-        <is>
-          <t>varchar(32) FK</t>
-        </is>
-      </c>
-      <c r="C6" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D6" s="84" t="inlineStr">
-        <is>
-          <t>Riferimento a learning_lezione.id.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="84" t="inlineStr">
-        <is>
-          <t>modalita</t>
-        </is>
-      </c>
-      <c r="B7" s="84" t="inlineStr">
-        <is>
-          <t>varchar(10)</t>
-        </is>
-      </c>
-      <c r="C7" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D7" s="84" t="inlineStr">
-        <is>
-          <t>guidato oppure finale. UNIQUE con lezione_id.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="84" t="inlineStr">
-        <is>
-          <t>titolo</t>
-        </is>
-      </c>
-      <c r="B8" s="84" t="inlineStr">
-        <is>
-          <t>varchar(160)</t>
-        </is>
-      </c>
-      <c r="C8" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D8" s="84" t="inlineStr">
-        <is>
-          <t>Titolo mostrato all'utente.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" style="40" min="1" max="1"/>
-    <col width="22" customWidth="1" style="40" min="2" max="2"/>
-    <col width="14" customWidth="1" style="40" min="3" max="3"/>
-    <col width="68" customWidth="1" style="40" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="81" t="inlineStr">
-        <is>
-          <t>STRUTTURA_QUIZ_GUIDATO — quesiti dell'esercizio guidato</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1" s="40">
-      <c r="A2" s="82" t="inlineStr">
-        <is>
-          <t>Tabella Neon: struttura_quiz_guidato, dalla separazione di learning_quesito. Correzione immediata, un quesito alla volta, senza punteggio. API: /api/lezioni/&lt;id&gt;/quiz/guidato/quesiti/&lt;qid&gt;/verifica/</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="83" t="inlineStr">
-        <is>
-          <t>Colonna</t>
-        </is>
-      </c>
-      <c r="B4" s="83" t="inlineStr">
-        <is>
-          <t>Tipo Neon</t>
-        </is>
-      </c>
-      <c r="C4" s="83" t="inlineStr">
-        <is>
-          <t>Obbligatoria</t>
-        </is>
-      </c>
-      <c r="D4" s="83" t="inlineStr">
-        <is>
-          <t>Descrizione</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="84" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B5" s="84" t="inlineStr">
-        <is>
-          <t>bigint (identity)</t>
-        </is>
-      </c>
-      <c r="C5" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D5" s="84" t="inlineStr">
-        <is>
-          <t>Chiave primaria tecnica. Univoca solo dentro questa tabella.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="84" t="inlineStr">
-        <is>
-          <t>quiz_id</t>
-        </is>
-      </c>
-      <c r="B6" s="84" t="inlineStr">
-        <is>
-          <t>bigint FK</t>
-        </is>
-      </c>
-      <c r="C6" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D6" s="84" t="inlineStr">
-        <is>
-          <t>Riferimento a struttura_quiz.id, modalita guidato.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="84" t="inlineStr">
-        <is>
-          <t>ordine</t>
-        </is>
-      </c>
-      <c r="B7" s="84" t="inlineStr">
-        <is>
-          <t>smallint</t>
-        </is>
-      </c>
-      <c r="C7" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D7" s="84" t="inlineStr">
-        <is>
-          <t>Posizione del quesito. UNIQUE con quiz_id.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="84" t="inlineStr">
-        <is>
-          <t>tipo</t>
-        </is>
-      </c>
-      <c r="B8" s="84" t="inlineStr">
-        <is>
-          <t>varchar(20)</t>
-        </is>
-      </c>
-      <c r="C8" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D8" s="84" t="inlineStr">
-        <is>
-          <t>completamento oppure scelta_multipla.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="84" t="inlineStr">
-        <is>
-          <t>testo</t>
-        </is>
-      </c>
-      <c r="B9" s="84" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C9" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D9" s="84" t="inlineStr">
-        <is>
-          <t>Testo del quesito mostrato all'utente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="84" t="inlineStr">
-        <is>
-          <t>opzioni</t>
-        </is>
-      </c>
-      <c r="B10" s="84" t="inlineStr">
-        <is>
-          <t>jsonb</t>
-        </is>
-      </c>
-      <c r="C10" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D10" s="84" t="inlineStr">
-        <is>
-          <t>Alternative per scelta_multipla; lista vuota per completamento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="84" t="inlineStr">
-        <is>
-          <t>risposta_corretta</t>
-        </is>
-      </c>
-      <c r="B11" s="84" t="inlineStr">
-        <is>
-          <t>varchar(300)</t>
-        </is>
-      </c>
-      <c r="C11" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D11" s="84" t="inlineStr">
-        <is>
-          <t>Soluzione. Varianti accettate separate da «|».</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="84" t="inlineStr">
-        <is>
-          <t>spiegazione</t>
-        </is>
-      </c>
-      <c r="B12" s="84" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C12" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D12" s="84" t="inlineStr">
-        <is>
-          <t>Mostrata dopo la verifica. Mai inviata al client prima della risposta.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" style="40" min="1" max="1"/>
-    <col width="22" customWidth="1" style="40" min="2" max="2"/>
-    <col width="14" customWidth="1" style="40" min="3" max="3"/>
-    <col width="68" customWidth="1" style="40" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="81" t="inlineStr">
-        <is>
-          <t>STRUTTURA_QUIZ_FINALE — quesiti del quiz finale</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1" s="40">
-      <c r="A2" s="82" t="inlineStr">
-        <is>
-          <t>Tabella Neon: struttura_quiz_finale, dalla separazione di learning_quesito. Corretti in blocco: producono il punteggio in learning_progresso (soglia 70). API: /api/lezioni/&lt;id&gt;/quiz/finale/quesiti/&lt;qid&gt;/verifica/</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="83" t="inlineStr">
-        <is>
-          <t>Colonna</t>
-        </is>
-      </c>
-      <c r="B4" s="83" t="inlineStr">
-        <is>
-          <t>Tipo Neon</t>
-        </is>
-      </c>
-      <c r="C4" s="83" t="inlineStr">
-        <is>
-          <t>Obbligatoria</t>
-        </is>
-      </c>
-      <c r="D4" s="83" t="inlineStr">
-        <is>
-          <t>Descrizione</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="84" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B5" s="84" t="inlineStr">
-        <is>
-          <t>bigint (identity)</t>
-        </is>
-      </c>
-      <c r="C5" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D5" s="84" t="inlineStr">
-        <is>
-          <t>Chiave primaria tecnica. Univoca solo dentro questa tabella.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="84" t="inlineStr">
-        <is>
-          <t>quiz_id</t>
-        </is>
-      </c>
-      <c r="B6" s="84" t="inlineStr">
-        <is>
-          <t>bigint FK</t>
-        </is>
-      </c>
-      <c r="C6" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D6" s="84" t="inlineStr">
-        <is>
-          <t>Riferimento a struttura_quiz.id, modalita finale.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="84" t="inlineStr">
-        <is>
-          <t>ordine</t>
-        </is>
-      </c>
-      <c r="B7" s="84" t="inlineStr">
-        <is>
-          <t>smallint</t>
-        </is>
-      </c>
-      <c r="C7" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D7" s="84" t="inlineStr">
-        <is>
-          <t>Posizione del quesito. UNIQUE con quiz_id.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="84" t="inlineStr">
-        <is>
-          <t>tipo</t>
-        </is>
-      </c>
-      <c r="B8" s="84" t="inlineStr">
-        <is>
-          <t>varchar(20)</t>
-        </is>
-      </c>
-      <c r="C8" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D8" s="84" t="inlineStr">
-        <is>
-          <t>completamento oppure scelta_multipla.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="84" t="inlineStr">
-        <is>
-          <t>testo</t>
-        </is>
-      </c>
-      <c r="B9" s="84" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C9" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D9" s="84" t="inlineStr">
-        <is>
-          <t>Testo del quesito mostrato all'utente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="84" t="inlineStr">
-        <is>
-          <t>opzioni</t>
-        </is>
-      </c>
-      <c r="B10" s="84" t="inlineStr">
-        <is>
-          <t>jsonb</t>
-        </is>
-      </c>
-      <c r="C10" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D10" s="84" t="inlineStr">
-        <is>
-          <t>Alternative per scelta_multipla; lista vuota per completamento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="84" t="inlineStr">
-        <is>
-          <t>risposta_corretta</t>
-        </is>
-      </c>
-      <c r="B11" s="84" t="inlineStr">
-        <is>
-          <t>varchar(300)</t>
-        </is>
-      </c>
-      <c r="C11" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D11" s="84" t="inlineStr">
-        <is>
-          <t>Soluzione. Varianti accettate separate da «|».</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="84" t="inlineStr">
-        <is>
-          <t>spiegazione</t>
-        </is>
-      </c>
-      <c r="B12" s="84" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C12" s="84" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D12" s="84" t="inlineStr">
-        <is>
-          <t>Mostrata dopo la verifica. Mai inviata al client prima della risposta.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" style="40" min="1" max="1"/>
-    <col width="34" customWidth="1" style="40" min="2" max="2"/>
-    <col width="46" customWidth="1" style="40" min="3" max="3"/>
-    <col width="74" customWidth="1" style="40" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="81" t="inlineStr">
-        <is>
-          <t>MODELLO DATI — corrispondenza fogli / tabelle Neon</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1" s="40">
-      <c r="A2" s="82" t="inlineStr">
-        <is>
-          <t>Stato dopo la migration learning.0006. Se una struttura cambia su Neon va aggiornata anche qui.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="83" t="inlineStr">
-        <is>
-          <t>Tabella Neon (attuale)</t>
-        </is>
-      </c>
-      <c r="B4" s="83" t="inlineStr">
-        <is>
-          <t>Nome precedente</t>
-        </is>
-      </c>
-      <c r="C4" s="83" t="inlineStr">
-        <is>
-          <t>Foglio di riferimento</t>
-        </is>
-      </c>
-      <c r="D4" s="83" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="84" t="inlineStr">
-        <is>
-          <t>mapping_area_lezione</t>
-        </is>
-      </c>
-      <c r="B5" s="84" t="inlineStr">
-        <is>
-          <t>learning_area</t>
-        </is>
-      </c>
-      <c r="C5" s="84" t="inlineStr">
-        <is>
-          <t>Liste (col. Area Didattica)</t>
-        </is>
-      </c>
-      <c r="D5" s="84" t="inlineStr">
-        <is>
-          <t>Rinominata: tabella di mapping codice→etichetta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="84" t="inlineStr">
-        <is>
-          <t>mapping_tipologia</t>
-        </is>
-      </c>
-      <c r="B6" s="84" t="inlineStr">
-        <is>
-          <t>learning_tipologia</t>
-        </is>
-      </c>
-      <c r="C6" s="84" t="inlineStr">
-        <is>
-          <t>Liste (col. Tipologia Lezione)</t>
-        </is>
-      </c>
-      <c r="D6" s="84" t="inlineStr">
-        <is>
-          <t>Rinominata.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="84" t="inlineStr">
-        <is>
-          <t>mapping_livello</t>
-        </is>
-      </c>
-      <c r="B7" s="84" t="inlineStr">
-        <is>
-          <t>learning_livello</t>
-        </is>
-      </c>
-      <c r="C7" s="84" t="inlineStr">
-        <is>
-          <t>Liste (col. Livello Linguistico)</t>
-        </is>
-      </c>
-      <c r="D7" s="84" t="inlineStr">
-        <is>
-          <t>Rinominata.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="84" t="inlineStr">
-        <is>
-          <t>mapping_difficolta_lezione</t>
-        </is>
-      </c>
-      <c r="B8" s="84" t="inlineStr">
-        <is>
-          <t>learning_difficolta</t>
-        </is>
-      </c>
-      <c r="C8" s="84" t="inlineStr">
-        <is>
-          <t>Liste (col. Difficoltà)</t>
-        </is>
-      </c>
-      <c r="D8" s="84" t="inlineStr">
-        <is>
-          <t>Rinominata, senza accento: un identificatore accentato andrebbe virgolettato in ogni query Postgres.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="84" t="inlineStr">
-        <is>
-          <t>learning_statolezione</t>
-        </is>
-      </c>
-      <c r="B9" s="84" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C9" s="84" t="inlineStr">
-        <is>
-          <t>Liste (col. Stato della Lezione)</t>
-        </is>
-      </c>
-      <c r="D9" s="84" t="inlineStr">
-        <is>
-          <t>Invariata: fuori dal perimetro del refactor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="84" t="inlineStr">
-        <is>
-          <t>learning_lezione</t>
-        </is>
-      </c>
-      <c r="B10" s="84" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C10" s="84" t="inlineStr">
-        <is>
-          <t>Programma Lezioni</t>
-        </is>
-      </c>
-      <c r="D10" s="84" t="inlineStr">
-        <is>
-          <t>Rimosse le colonne priorita e importanza_mvp_id.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="84" t="inlineStr">
-        <is>
-          <t>learning_prerequisito</t>
-        </is>
-      </c>
-      <c r="B11" s="84" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C11" s="84" t="inlineStr">
-        <is>
-          <t>Programma Lezioni (Prerequisiti) e Percorso MVP (Dipendenze)</t>
-        </is>
-      </c>
-      <c r="D11" s="84" t="inlineStr">
-        <is>
-          <t>MANTENUTA: vedi nota in fondo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="84" t="inlineStr">
-        <is>
-          <t>struttura_lezione</t>
-        </is>
-      </c>
-      <c r="B12" s="84" t="inlineStr">
-        <is>
-          <t>learning_sezionelezione</t>
-        </is>
-      </c>
-      <c r="C12" s="84" t="inlineStr">
-        <is>
-          <t>Struttura_Lezione</t>
-        </is>
-      </c>
-      <c r="D12" s="84" t="inlineStr">
-        <is>
-          <t>Rinominata: è la struttura della lezione.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="84" t="inlineStr">
-        <is>
-          <t>struttura_quiz</t>
-        </is>
-      </c>
-      <c r="B13" s="84" t="inlineStr">
-        <is>
-          <t>learning_quiz</t>
-        </is>
-      </c>
-      <c r="C13" s="84" t="inlineStr">
-        <is>
-          <t>Struttura_Quiz</t>
-        </is>
-      </c>
-      <c r="D13" s="84" t="inlineStr">
-        <is>
-          <t>Rinominata.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="84" t="inlineStr">
-        <is>
-          <t>struttura_quiz_guidato</t>
-        </is>
-      </c>
-      <c r="B14" s="84" t="inlineStr">
-        <is>
-          <t>learning_quesito (parte guidata)</t>
-        </is>
-      </c>
-      <c r="C14" s="84" t="inlineStr">
-        <is>
-          <t>struttura_quiz_guidato</t>
-        </is>
-      </c>
-      <c r="D14" s="84" t="inlineStr">
-        <is>
-          <t>Nuova, da separazione di learning_quesito.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="84" t="inlineStr">
-        <is>
-          <t>struttura_quiz_finale</t>
-        </is>
-      </c>
-      <c r="B15" s="84" t="inlineStr">
-        <is>
-          <t>learning_quesito (parte finale)</t>
-        </is>
-      </c>
-      <c r="C15" s="84" t="inlineStr">
-        <is>
-          <t>struttura_quiz_finale</t>
-        </is>
-      </c>
-      <c r="D15" s="84" t="inlineStr">
-        <is>
-          <t>Nuova, da separazione di learning_quesito.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="84" t="inlineStr">
-        <is>
-          <t>learning_progresso</t>
-        </is>
-      </c>
-      <c r="B16" s="84" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C16" s="84" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D16" s="84" t="inlineStr">
-        <is>
-          <t>Invariata. Popolata dagli utenti, non dal workbook.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="84" t="inlineStr">
-        <is>
-          <t>learning_user</t>
-        </is>
-      </c>
-      <c r="B17" s="84" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C17" s="84" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D17" s="84" t="inlineStr">
-        <is>
-          <t>Invariata.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="84" t="inlineStr">
-        <is>
-          <t>learning_importanza</t>
-        </is>
-      </c>
-      <c r="B18" s="84" t="inlineStr">
-        <is>
-          <t>learning_importanza</t>
-        </is>
-      </c>
-      <c r="C18" s="84" t="inlineStr">
-        <is>
-          <t>— (eliminata)</t>
-        </is>
-      </c>
-      <c r="D18" s="84" t="inlineStr">
-        <is>
-          <t>ELIMINATA con la colonna learning_lezione.priorita.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="85" t="inlineStr">
-        <is>
-          <t>Perché learning_prerequisito non è stata eliminata</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="84" t="inlineStr">
-        <is>
-          <t>La regola «ultime cifre dell'ID meno 1» e' stata verificata su tutti i 119 archi esistenti: riproduce il dato esattamente in 64 casi su 96. Non copre 22 lezioni con piu' di un prerequisito, 18 archi fra aree diverse (COM-A1-001 richiede GRA-A1-003) e 15 lezioni con suffisso -001 (genererebbe -000, inesistente); in un caso inverte la dipendenza (COM-A1-002 richiede COM-A1-004). Eliminare la tabella avrebbe perso 55 archi su 119 e reso inutilizzabile la validazione del DAG in services.py. La logica e' comunque disponibile come campo derivato Lezione.prerequisito_derivato, esposto in API e mostrato nel frontend come «Segue X», senza impatti sullo schema.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A21:D25"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:B20"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="30" customWidth="1" style="39" min="1" max="1"/>
-    <col width="120" customWidth="1" style="39" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="18" customHeight="1" s="40">
-      <c r="A1" s="41" t="inlineStr">
-        <is>
-          <t>LOGICA DIDATTICA</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="15" customHeight="1" s="40">
-      <c r="A2" s="42" t="inlineStr">
-        <is>
-          <t>Le scelte progettuali alla base della nuova struttura del programma.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="42" customHeight="1" s="40">
-      <c r="A4" s="62" t="inlineStr">
-        <is>
-          <t>1. Categorie scelte</t>
-        </is>
-      </c>
-      <c r="B4" s="63" t="inlineStr">
-        <is>
-          <t>Tre aree didattiche: GRAMMATICA (il sistema della lingua), VOCABOLARIO (le parole e le combinazioni) e COMUNICAZIONE (l'uso reale della lingua). Ogni area ha un codice ID (GRA, VOC, COM), un colore e un template di pagina dedicato.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="97.5" customHeight="1" s="40">
-      <c r="A6" s="62" t="inlineStr">
-        <is>
-          <t>2. Perché Dialogo e Produzione sono state unite</t>
-        </is>
-      </c>
-      <c r="B6" s="63" t="inlineStr">
-        <is>
-          <t>Le vecchie categorie Dialogo e Produzione si sovrapponevano: entrambe allenavano la produzione orale e la differenza (conversazione a due vs. monologo/testo) è una differenza di FORMATO dell'attività, non di area didattica. Sono state quindi unite nell'area COMUNICAZIONE, e la distinzione è diventata una «Tipologia Lezione» interna con tre valori: DIALOGO (comprensione + interazione guidata in uno scenario), PRODUZIONE GUIDATA (lo studente produce con modello e traccia) e PRODUZIONE LIBERA (lo studente produce in autonomia con feedback). Questo realizza la distinzione didatticamente corretta comprensione → produzione guidata → produzione libera, senza moltiplicare le sezioni della Web App: nel menu l'utente vede una sola area «Comunicazione».</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="84" customHeight="1" s="40">
-      <c r="A8" s="62" t="inlineStr">
-        <is>
-          <t>3. Categorie eliminate o reintegrate</t>
-        </is>
-      </c>
-      <c r="B8" s="63" t="inlineStr">
-        <is>
-          <t>Speaking e Scrittura NON tornano come categorie separate: sono competenze trasversali, tracciate nella colonna «Competenze Allenate» (ogni lezione di Comunicazione indica se allena speaking, scrittura o entrambi).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="84" customHeight="1" s="40">
-      <c r="A10" s="62" t="inlineStr">
-        <is>
-          <t>4. Progressione da A1 a C1</t>
-        </is>
-      </c>
-      <c r="B10" s="63" t="inlineStr">
-        <is>
-          <t>Ogni livello CEFR è un «capitolo» del percorso. Dentro ogni livello le lezioni si alternano secondo il ciclo: strumenti (grammatica + lessico) → applicazione (dialogo) → produzione guidata → produzione libera. La colonna «Ordine nel Percorso» definisce la sequenza consigliata unica (1-104); «Lezione Precedente/Successiva» la rendono navigabile; «Prerequisiti» elenca le dipendenze reali (che possono attraversare le aree: es. il dialogo «Raccontare il weekend» richiede il past simple). La difficoltà è ricalibrata ALL'INTERNO di ogni livello (una lezione A1 «Alta» resta più facile di una B2 «Bassa»).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="55.5" customHeight="1" s="40">
-      <c r="A12" s="62" t="inlineStr">
-        <is>
-          <t>5. Collegamento tra grammatica, vocabolario e comunicazione</t>
-        </is>
-      </c>
-      <c r="B12" s="63" t="inlineStr">
-        <is>
-          <t>Regola dei blocchi: prima si insegnano gli strumenti (GRA/VOC), poi si usano in uno scenario (COM-Dialogo), poi si produce (COM-Produzione). Esempio A1: to be → «Presentarsi e salutare» (dialogo) → «Parlare di sé» (produzione guidata). Ogni lezione COM dichiara nei prerequisiti le lezioni GRA/VOC necessarie, così la Web App può bloccare o consigliare le lezioni nell'ordine giusto con una semplice logica a dipendenze.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="55.5" customHeight="1" s="40">
-      <c r="A14" s="62" t="inlineStr">
-        <is>
-          <t>6. Come si evitano le sovrapposizioni</t>
-        </is>
-      </c>
-      <c r="B14" s="63" t="inlineStr">
-        <is>
-          <t>Speaking, Scrittura, Dialogo e Produzione non sono più categorie parallele ma tre livelli distinti del modello dati: AREA (dove sta la lezione nel menu) → TIPOLOGIA (che formato ha l'attività) → COMPETENZE (cosa allena). Una lezione appartiene a una sola area e a una sola tipologia, ma può allenare più competenze. Questo elimina ogni ambiguità di classificazione.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="55.5" customHeight="1" s="40">
-      <c r="A16" s="62" t="inlineStr">
-        <is>
-          <t>7. Focus sugli studenti italiani</t>
-        </is>
-      </c>
-      <c r="B16" s="63" t="inlineStr">
-        <is>
-          <t>Ogni lezione ha la colonna «Errori Tipici degli Italiani» con calchi, falsi amici e interferenze specifiche (I have 25 years, informations, I am agree, in Monday, listen music...). Sono state aggiunte lezioni che esistono SOLO in ottica italiana: falsi amici (A1 e B1), preposizioni in/on/at, articoli avanzati e omissione, verbi+preposizioni.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="97.5" customHeight="1" s="40">
-      <c r="A18" s="62" t="inlineStr">
-        <is>
-          <t>8. Correzioni principali rispetto alla bozza</t>
-        </is>
-      </c>
-      <c r="B18" s="63" t="inlineStr">
-        <is>
-          <t>a) Aggiunto il PRESENT CONTINUOUS, assente nella bozza pur essendo obbligatorio in A1, con lezione di contrasto simple/continuous. b) Aggiunte 8 lezioni A1 mancanti (possessivi, dimostrativi, question words, can, preposizioni, avverbi di frequenza...). c) Il Vocabolario passa da 3 a 17 lezioni: era sottodimensionato rispetto al suo peso didattico. d) Aggiunta la negativa/interrogativa del past simple (mancava). e) Riequilibrate le difficoltà (es. «to be negativa» da Media a Bassa; «present simple vs continuous» ad Alta). f) Aggiunti scenari comunicativi mancanti (negozio, reclami, e-mail semplice in A2). g) Descrizioni differenziate per tipologia invece del testo fotocopia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="55.5" customHeight="1" s="40">
-      <c r="A20" s="62" t="inlineStr">
-        <is>
-          <t>9. Struttura minima per l'MVP</t>
-        </is>
-      </c>
-      <c r="B20" s="63" t="inlineStr">
-        <is>
-          <t>MVP = solo livello A1 con le 3 aree già presenti ma in versione ridotta: ~26 lezioni (vedi foglio «Percorso MVP»). Funzionalità minime: pagina-lezione secondo i template, quiz a scelta multipla/completamento, percorso lineare con blocco sui prerequisiti, salvataggio dei progressi. Rimandate a fasi successive: feedback automatico sulla produzione libera, spaced repetition del lessico.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10765,7 +9419,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="27.75" customHeight="1" s="40">
       <c r="A4" s="44" t="inlineStr">
         <is>
@@ -11916,302 +10569,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:H9"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="16" customWidth="1" style="39" min="1" max="1"/>
-    <col width="34" customWidth="1" style="39" min="2" max="2"/>
-    <col width="44" customWidth="1" style="39" min="3" max="3"/>
-    <col width="26" customWidth="1" style="39" min="4" max="4"/>
-    <col width="52" customWidth="1" style="39" min="5" max="5"/>
-    <col width="10" customWidth="1" style="39" min="6" max="6"/>
-    <col width="11" customWidth="1" style="39" min="7" max="7"/>
-    <col width="30" customWidth="1" style="39" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="18" customHeight="1" s="40">
-      <c r="A1" s="41" t="inlineStr">
-        <is>
-          <t>ROADMAP DI SVILUPPO</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="15" customHeight="1" s="40">
-      <c r="A2" s="42" t="inlineStr">
-        <is>
-          <t>Cinque fasi incrementali: ogni fase produce una app utilizzabile e più completa della precedente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="27.75" customHeight="1" s="40">
-      <c r="A4" s="44" t="inlineStr">
-        <is>
-          <t>Fase</t>
-        </is>
-      </c>
-      <c r="B4" s="44" t="inlineStr">
-        <is>
-          <t>Obiettivo</t>
-        </is>
-      </c>
-      <c r="C4" s="44" t="inlineStr">
-        <is>
-          <t>Lezioni da Sviluppare</t>
-        </is>
-      </c>
-      <c r="D4" s="44" t="inlineStr">
-        <is>
-          <t>Categorie Coinvolte</t>
-        </is>
-      </c>
-      <c r="E4" s="44" t="inlineStr">
-        <is>
-          <t>Funzionalità Necessarie</t>
-        </is>
-      </c>
-      <c r="F4" s="44" t="inlineStr">
-        <is>
-          <t>Priorità</t>
-        </is>
-      </c>
-      <c r="G4" s="44" t="inlineStr">
-        <is>
-          <t>Complessità</t>
-        </is>
-      </c>
-      <c r="H4" s="44" t="inlineStr">
-        <is>
-          <t>Dipendenze</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="67.5" customHeight="1" s="40">
-      <c r="A5" s="69" t="inlineStr">
-        <is>
-          <t>Fase 1 — MVP</t>
-        </is>
-      </c>
-      <c r="B5" s="56" t="inlineStr">
-        <is>
-          <t>Percorso A1 completo e utilizzabile «da zero alla prima conversazione».</t>
-        </is>
-      </c>
-      <c r="C5" s="56" t="inlineStr">
-        <is>
-          <t>Le 26 lezioni del foglio «Percorso MVP» (partendo dalle 12 Essenziali).</t>
-        </is>
-      </c>
-      <c r="D5" s="56" t="inlineStr">
-        <is>
-          <t>Grammatica, Vocabolario, Comunicazione</t>
-        </is>
-      </c>
-      <c r="E5" s="56" t="inlineStr">
-        <is>
-          <t>Pagina-lezione secondo i 3 template; quiz a scelta multipla e completamento; percorso lineare con blocco sui prerequisiti; salvataggio progressi.</t>
-        </is>
-      </c>
-      <c r="F5" s="57" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="G5" s="55" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="H5" s="56" t="inlineStr">
-        <is>
-          <t>Nessuna</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="67.5" customHeight="1" s="40">
-      <c r="A6" s="69" t="inlineStr">
-        <is>
-          <t>Fase 2 — Ampliamento A1-A2</t>
-        </is>
-      </c>
-      <c r="B6" s="56" t="inlineStr">
-        <is>
-          <t>Coprire integralmente i livelli A1 e A2 (56 lezioni totali).</t>
-        </is>
-      </c>
-      <c r="C6" s="56" t="inlineStr">
-        <is>
-          <t>Le lezioni A1 rimanenti (Secondarie) e tutte le 25 lezioni A2.</t>
-        </is>
-      </c>
-      <c r="D6" s="56" t="inlineStr">
-        <is>
-          <t>Tutte e tre le aree</t>
-        </is>
-      </c>
-      <c r="E6" s="56" t="inlineStr">
-        <is>
-          <t>Esercizi di riordino frase e abbinamento; dettati brevi; ripasso programmato del lessico (spaced repetition); statistiche di avanzamento per area.</t>
-        </is>
-      </c>
-      <c r="F6" s="57" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="G6" s="55" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="H6" s="56" t="inlineStr">
-        <is>
-          <t>Fase 1 completata</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="67.5" customHeight="1" s="40">
-      <c r="A7" s="69" t="inlineStr">
-        <is>
-          <t>Fase 3 — Introduzione B1</t>
-        </is>
-      </c>
-      <c r="B7" s="56" t="inlineStr">
-        <is>
-          <t>Aprire il livello intermedio con test d'ingresso.</t>
-        </is>
-      </c>
-      <c r="C7" s="56" t="inlineStr">
-        <is>
-          <t>Le 22 lezioni B1 (priorità: present perfect vs past simple, tempi narrativi, phrasal verbs, colloquio di lavoro).</t>
-        </is>
-      </c>
-      <c r="D7" s="56" t="inlineStr">
-        <is>
-          <t>Tutte e tre le aree</t>
-        </is>
-      </c>
-      <c r="E7" s="56" t="inlineStr">
-        <is>
-          <t>Test di livello iniziale; produzione scritta con auto-valutazione guidata (checklist); registrazione vocale per lo speaking; certificato di completamento livello.</t>
-        </is>
-      </c>
-      <c r="F7" s="55" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G7" s="57" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="H7" s="56" t="inlineStr">
-        <is>
-          <t>Fase 2 completata</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="67.5" customHeight="1" s="40">
-      <c r="A8" s="69" t="inlineStr">
-        <is>
-          <t>Fase 4 — Ampliamento B2-C1</t>
-        </is>
-      </c>
-      <c r="B8" s="56" t="inlineStr">
-        <is>
-          <t>Completare il percorso fino al livello avanzato.</t>
-        </is>
-      </c>
-      <c r="C8" s="56" t="inlineStr">
-        <is>
-          <t>Le 15 lezioni B2 e le 11 lezioni C1.</t>
-        </is>
-      </c>
-      <c r="D8" s="56" t="inlineStr">
-        <is>
-          <t>Grammatica, Vocabolario, Comunicazione</t>
-        </is>
-      </c>
-      <c r="E8" s="56" t="inlineStr">
-        <is>
-          <t>Feedback AI sulla produzione libera (scritta e orale); simulazioni di dialogo a risposta aperta; percorsi tematici (Business English, Travel).</t>
-        </is>
-      </c>
-      <c r="F8" s="55" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G8" s="57" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="H8" s="56" t="inlineStr">
-        <is>
-          <t>Fase 3 completata</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="67.5" customHeight="1" s="40">
-      <c r="A9" s="69" t="inlineStr">
-        <is>
-          <t>Fase 5 — Funzionalità avanzate</t>
-        </is>
-      </c>
-      <c r="B9" s="56" t="inlineStr">
-        <is>
-          <t>Fidelizzazione e personalizzazione dell'apprendimento.</t>
-        </is>
-      </c>
-      <c r="C9" s="56" t="inlineStr">
-        <is>
-          <t>Nessuna nuova lezione: consolidamento e contenuti extra (lezioni stagionali, cultura).</t>
-        </is>
-      </c>
-      <c r="D9" s="56" t="inlineStr">
-        <is>
-          <t>Trasversale</t>
-        </is>
-      </c>
-      <c r="E9" s="56" t="inlineStr">
-        <is>
-          <t>Percorsi adattivi basati sugli errori dell'utente; gamification (streak, badge, classifiche); modalità ripasso rapido; app offline; notifiche intelligenti.</t>
-        </is>
-      </c>
-      <c r="F9" s="49" t="inlineStr">
-        <is>
-          <t>Bassa</t>
-        </is>
-      </c>
-      <c r="G9" s="57" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="H9" s="56" t="inlineStr">
-        <is>
-          <t>Fasi 1-4; base utenti attiva</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14429,7 +12787,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15277,7 +13635,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -16381,7 +14739,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -16403,11 +14761,10 @@
     <row r="2" ht="15" customHeight="1" s="40">
       <c r="A2" s="42" t="inlineStr">
         <is>
-          <t>Queste colonne alimentano le convalide dati degli altri fogli. Ogni colonna corrisponde a una tabella su Neon: Area Didattica → mapping_area_lezione, Tipologia Lezione → mapping_tipologia, Livello Linguistico → mapping_livello, Difficoltà → mapping_difficolta_lezione, Stato della Lezione → learning_statolezione.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Queste colonne alimentano le convalide dati degli altri fogli. Ogni colonna corrisponde a una tabella su Neon: Area Didattica → dim_area_lezione, Tipologia Lezione → dim_tipologia, Livello Linguistico → dim_livello, Difficoltà → dim_difficolta_lezione, Stato della Lezione → dim_stato_lezione.</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="15" customHeight="1" s="40">
       <c r="A4" s="44" t="inlineStr">
         <is>
@@ -16604,9 +14961,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
     <row r="14" ht="15" customHeight="1" s="40">
       <c r="A14" s="75" t="inlineStr">
         <is>
@@ -16666,7 +15020,6 @@
       <c r="A19" s="80" t="n"/>
       <c r="B19" s="53" t="n"/>
     </row>
-    <row r="20"/>
     <row r="21" ht="15" customHeight="1" s="40">
       <c r="A21" s="42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Normalizzato problema lezione GRA-008 e prodotto documenti .MD di lettura progetto
</commit_message>
<xml_diff>
--- a/programma_lezioni_inglese_no_audio.xlsx
+++ b/programma_lezioni_inglese_no_audio.xlsx
@@ -734,8 +734,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TabMVP" displayName="TabMVP" ref="A4:I32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A4:I32"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TabMVP" displayName="TabMVP" ref="A4:I33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A4:I33"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Ordine MVP"/>
     <tableColumn id="2" name="ID Lezione"/>
@@ -9391,7 +9391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="39" min="1" max="1"/>
@@ -9847,12 +9847,12 @@
       </c>
       <c r="B15" s="46" t="inlineStr">
         <is>
-          <t>GRA-A1-009</t>
+          <t>GRA-A1-008</t>
         </is>
       </c>
       <c r="C15" s="56" t="inlineStr">
         <is>
-          <t>There is e there are</t>
+          <t>Dimostrativi: this, that, these, those</t>
         </is>
       </c>
       <c r="D15" s="47" t="inlineStr">
@@ -9867,16 +9867,16 @@
       </c>
       <c r="F15" s="56" t="inlineStr">
         <is>
-          <t>«C'è/ci sono» è tra le prime strutture richieste nelle descrizioni.</t>
+          <t>Indicare oggetti e persone vicini o lontani: prerequisito diretto di there is/there are.</t>
         </is>
       </c>
       <c r="G15" s="56" t="inlineStr">
         <is>
-          <t>GRA-A1-008</t>
+          <t>GRA-A1-007</t>
         </is>
       </c>
       <c r="H15" s="46" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="40">
@@ -9885,17 +9885,17 @@
       </c>
       <c r="B16" s="46" t="inlineStr">
         <is>
-          <t>VOC-A1-003</t>
+          <t>GRA-A1-009</t>
         </is>
       </c>
       <c r="C16" s="56" t="inlineStr">
         <is>
-          <t>Casa e oggetti quotidiani</t>
-        </is>
-      </c>
-      <c r="D16" s="54" t="inlineStr">
-        <is>
-          <t>Vocabolario</t>
+          <t>There is e there are</t>
+        </is>
+      </c>
+      <c r="D16" s="47" t="inlineStr">
+        <is>
+          <t>Grammatica</t>
         </is>
       </c>
       <c r="E16" s="49" t="inlineStr">
@@ -9905,16 +9905,16 @@
       </c>
       <c r="F16" s="56" t="inlineStr">
         <is>
-          <t>Lessico descrittivo espandibile in seguito senza bloccare il percorso.</t>
+          <t>«C'è/ci sono» è tra le prime strutture richieste nelle descrizioni.</t>
         </is>
       </c>
       <c r="G16" s="56" t="inlineStr">
         <is>
-          <t>VOC-A1-002</t>
+          <t>GRA-A1-008</t>
         </is>
       </c>
       <c r="H16" s="46" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="40">
@@ -9923,17 +9923,17 @@
       </c>
       <c r="B17" s="46" t="inlineStr">
         <is>
-          <t>GRA-A1-010</t>
+          <t>VOC-A1-003</t>
         </is>
       </c>
       <c r="C17" s="56" t="inlineStr">
         <is>
-          <t>Have got per possesso e caratteristiche</t>
-        </is>
-      </c>
-      <c r="D17" s="47" t="inlineStr">
-        <is>
-          <t>Grammatica</t>
+          <t>Casa e oggetti quotidiani</t>
+        </is>
+      </c>
+      <c r="D17" s="54" t="inlineStr">
+        <is>
+          <t>Vocabolario</t>
         </is>
       </c>
       <c r="E17" s="49" t="inlineStr">
@@ -9943,16 +9943,16 @@
       </c>
       <c r="F17" s="56" t="inlineStr">
         <is>
-          <t>Utile ma parzialmente sostituibile con have: può slittare alla Fase 2.</t>
+          <t>Lessico descrittivo espandibile in seguito senza bloccare il percorso.</t>
         </is>
       </c>
       <c r="G17" s="56" t="inlineStr">
         <is>
-          <t>GRA-A1-009</t>
+          <t>VOC-A1-002</t>
         </is>
       </c>
       <c r="H17" s="46" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="40">
@@ -9961,12 +9961,12 @@
       </c>
       <c r="B18" s="46" t="inlineStr">
         <is>
-          <t>GRA-A1-011</t>
+          <t>GRA-A1-010</t>
         </is>
       </c>
       <c r="C18" s="56" t="inlineStr">
         <is>
-          <t>Present simple: forma affermativa</t>
+          <t>Have got per possesso e caratteristiche</t>
         </is>
       </c>
       <c r="D18" s="47" t="inlineStr">
@@ -9981,12 +9981,12 @@
       </c>
       <c r="F18" s="56" t="inlineStr">
         <is>
-          <t>Il present simple è il cuore del livello A1; la -s è l'errore n.1 degli italiani.</t>
+          <t>Utile ma parzialmente sostituibile con have: può slittare alla Fase 2.</t>
         </is>
       </c>
       <c r="G18" s="56" t="inlineStr">
         <is>
-          <t>GRA-A1-010</t>
+          <t>GRA-A1-009</t>
         </is>
       </c>
       <c r="H18" s="46" t="n">
@@ -9999,12 +9999,12 @@
       </c>
       <c r="B19" s="46" t="inlineStr">
         <is>
-          <t>GRA-A1-012</t>
+          <t>GRA-A1-011</t>
         </is>
       </c>
       <c r="C19" s="56" t="inlineStr">
         <is>
-          <t>Present simple: negazioni e domande con do/does</t>
+          <t>Present simple: forma affermativa</t>
         </is>
       </c>
       <c r="D19" s="47" t="inlineStr">
@@ -10019,12 +10019,12 @@
       </c>
       <c r="F19" s="56" t="inlineStr">
         <is>
-          <t>Do/does è il primo vero scoglio strutturale: senza, nessuna domanda è possibile.</t>
+          <t>Il present simple è il cuore del livello A1; la -s è l'errore n.1 degli italiani.</t>
         </is>
       </c>
       <c r="G19" s="56" t="inlineStr">
         <is>
-          <t>GRA-A1-011</t>
+          <t>GRA-A1-010</t>
         </is>
       </c>
       <c r="H19" s="46" t="n">
@@ -10037,12 +10037,12 @@
       </c>
       <c r="B20" s="46" t="inlineStr">
         <is>
-          <t>GRA-A1-013</t>
+          <t>GRA-A1-012</t>
         </is>
       </c>
       <c r="C20" s="56" t="inlineStr">
         <is>
-          <t>Gli avverbi di frequenza e la loro posizione</t>
+          <t>Present simple: negazioni e domande con do/does</t>
         </is>
       </c>
       <c r="D20" s="47" t="inlineStr">
@@ -10057,16 +10057,16 @@
       </c>
       <c r="F20" s="56" t="inlineStr">
         <is>
-          <t>La posizione degli avverbi consolida il present simple con poco sforzo.</t>
+          <t>Do/does è il primo vero scoglio strutturale: senza, nessuna domanda è possibile.</t>
         </is>
       </c>
       <c r="G20" s="56" t="inlineStr">
         <is>
-          <t>GRA-A1-012</t>
+          <t>GRA-A1-011</t>
         </is>
       </c>
       <c r="H20" s="46" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="40">
@@ -10075,17 +10075,17 @@
       </c>
       <c r="B21" s="46" t="inlineStr">
         <is>
-          <t>COM-A1-004</t>
+          <t>GRA-A1-013</t>
         </is>
       </c>
       <c r="C21" s="56" t="inlineStr">
         <is>
-          <t>Parlare di sé: chi sono, cosa faccio</t>
-        </is>
-      </c>
-      <c r="D21" s="51" t="inlineStr">
-        <is>
-          <t>Comunicazione</t>
+          <t>Gli avverbi di frequenza e la loro posizione</t>
+        </is>
+      </c>
+      <c r="D21" s="47" t="inlineStr">
+        <is>
+          <t>Grammatica</t>
         </is>
       </c>
       <c r="E21" s="49" t="inlineStr">
@@ -10095,16 +10095,16 @@
       </c>
       <c r="F21" s="56" t="inlineStr">
         <is>
-          <t>Prima produzione personale: chiude il ciclo capire → imitare → produrre.</t>
+          <t>La posizione degli avverbi consolida il present simple con poco sforzo.</t>
         </is>
       </c>
       <c r="G21" s="56" t="inlineStr">
         <is>
-          <t>COM-A1-001, GRA-A1-003</t>
+          <t>GRA-A1-012</t>
         </is>
       </c>
       <c r="H21" s="46" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" ht="23.25" customHeight="1" s="40">
@@ -10113,17 +10113,17 @@
       </c>
       <c r="B22" s="46" t="inlineStr">
         <is>
-          <t>GRA-A1-014</t>
+          <t>COM-A1-004</t>
         </is>
       </c>
       <c r="C22" s="56" t="inlineStr">
         <is>
-          <t>Le question words: who, what, where, when, why, how</t>
-        </is>
-      </c>
-      <c r="D22" s="47" t="inlineStr">
-        <is>
-          <t>Grammatica</t>
+          <t>Parlare di sé: chi sono, cosa faccio</t>
+        </is>
+      </c>
+      <c r="D22" s="51" t="inlineStr">
+        <is>
+          <t>Comunicazione</t>
         </is>
       </c>
       <c r="E22" s="49" t="inlineStr">
@@ -10133,16 +10133,16 @@
       </c>
       <c r="F22" s="56" t="inlineStr">
         <is>
-          <t>Le wh-questions moltiplicano le capacità comunicative con una sola lezione.</t>
+          <t>Prima produzione personale: chiude il ciclo capire → imitare → produrre.</t>
         </is>
       </c>
       <c r="G22" s="56" t="inlineStr">
         <is>
-          <t>GRA-A1-013</t>
+          <t>COM-A1-001, GRA-A1-003</t>
         </is>
       </c>
       <c r="H22" s="46" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23" ht="27.75" customHeight="1" s="40">
@@ -10151,12 +10151,12 @@
       </c>
       <c r="B23" s="46" t="inlineStr">
         <is>
-          <t>GRA-A1-015</t>
+          <t>GRA-A1-014</t>
         </is>
       </c>
       <c r="C23" s="56" t="inlineStr">
         <is>
-          <t>Can e can't: abilità, permesso e richieste</t>
+          <t>Le question words: who, what, where, when, why, how</t>
         </is>
       </c>
       <c r="D23" s="47" t="inlineStr">
@@ -10171,16 +10171,16 @@
       </c>
       <c r="F23" s="56" t="inlineStr">
         <is>
-          <t>Can è semplice, subito spendibile nei dialoghi (richieste al bar, permessi).</t>
+          <t>Le wh-questions moltiplicano le capacità comunicative con una sola lezione.</t>
         </is>
       </c>
       <c r="G23" s="56" t="inlineStr">
         <is>
-          <t>GRA-A1-014</t>
+          <t>GRA-A1-013</t>
         </is>
       </c>
       <c r="H23" s="46" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="40">
@@ -10189,17 +10189,17 @@
       </c>
       <c r="B24" s="46" t="inlineStr">
         <is>
-          <t>COM-A1-002</t>
+          <t>GRA-A1-015</t>
         </is>
       </c>
       <c r="C24" s="56" t="inlineStr">
         <is>
-          <t>Al bar: ordinare da bere e da mangiare</t>
-        </is>
-      </c>
-      <c r="D24" s="51" t="inlineStr">
-        <is>
-          <t>Comunicazione</t>
+          <t>Can e can't: abilità, permesso e richieste</t>
+        </is>
+      </c>
+      <c r="D24" s="47" t="inlineStr">
+        <is>
+          <t>Grammatica</t>
         </is>
       </c>
       <c r="E24" s="49" t="inlineStr">
@@ -10209,16 +10209,16 @@
       </c>
       <c r="F24" s="56" t="inlineStr">
         <is>
-          <t>Scenario ad alta frequenza d'uso; dimostra il valore pratico della app.</t>
+          <t>Can è semplice, subito spendibile nei dialoghi (richieste al bar, permessi).</t>
         </is>
       </c>
       <c r="G24" s="56" t="inlineStr">
         <is>
-          <t>COM-A1-004, GRA-A1-015</t>
+          <t>GRA-A1-014</t>
         </is>
       </c>
       <c r="H24" s="46" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="40">
@@ -10227,17 +10227,17 @@
       </c>
       <c r="B25" s="46" t="inlineStr">
         <is>
-          <t>VOC-A1-004</t>
+          <t>COM-A1-002</t>
         </is>
       </c>
       <c r="C25" s="56" t="inlineStr">
         <is>
-          <t>Cibo, bevande e pasti</t>
-        </is>
-      </c>
-      <c r="D25" s="54" t="inlineStr">
-        <is>
-          <t>Vocabolario</t>
+          <t>Al bar: ordinare da bere e da mangiare</t>
+        </is>
+      </c>
+      <c r="D25" s="51" t="inlineStr">
+        <is>
+          <t>Comunicazione</t>
         </is>
       </c>
       <c r="E25" s="49" t="inlineStr">
@@ -10247,16 +10247,16 @@
       </c>
       <c r="F25" s="56" t="inlineStr">
         <is>
-          <t>Sinergico con lo scenario bar/ristorante ma non bloccante.</t>
+          <t>Scenario ad alta frequenza d'uso; dimostra il valore pratico della app.</t>
         </is>
       </c>
       <c r="G25" s="56" t="inlineStr">
         <is>
-          <t>VOC-A1-003</t>
+          <t>COM-A1-004, GRA-A1-015</t>
         </is>
       </c>
       <c r="H25" s="46" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="40">
@@ -10265,17 +10265,17 @@
       </c>
       <c r="B26" s="46" t="inlineStr">
         <is>
-          <t>GRA-A1-016</t>
+          <t>VOC-A1-004</t>
         </is>
       </c>
       <c r="C26" s="56" t="inlineStr">
         <is>
-          <t>Le preposizioni di tempo e luogo: in, on, at</t>
-        </is>
-      </c>
-      <c r="D26" s="47" t="inlineStr">
-        <is>
-          <t>Grammatica</t>
+          <t>Cibo, bevande e pasti</t>
+        </is>
+      </c>
+      <c r="D26" s="54" t="inlineStr">
+        <is>
+          <t>Vocabolario</t>
         </is>
       </c>
       <c r="E26" s="49" t="inlineStr">
@@ -10285,16 +10285,16 @@
       </c>
       <c r="F26" s="56" t="inlineStr">
         <is>
-          <t>In/on/at: l'area con più interferenza dall'italiano, serve dall'inizio.</t>
+          <t>Sinergico con lo scenario bar/ristorante ma non bloccante.</t>
         </is>
       </c>
       <c r="G26" s="56" t="inlineStr">
         <is>
-          <t>GRA-A1-015</t>
+          <t>VOC-A1-003</t>
         </is>
       </c>
       <c r="H26" s="46" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="40">
@@ -10303,17 +10303,17 @@
       </c>
       <c r="B27" s="46" t="inlineStr">
         <is>
-          <t>COM-A1-003</t>
+          <t>GRA-A1-016</t>
         </is>
       </c>
       <c r="C27" s="56" t="inlineStr">
         <is>
-          <t>In hotel: fare il check-in</t>
-        </is>
-      </c>
-      <c r="D27" s="51" t="inlineStr">
-        <is>
-          <t>Comunicazione</t>
+          <t>Le preposizioni di tempo e luogo: in, on, at</t>
+        </is>
+      </c>
+      <c r="D27" s="47" t="inlineStr">
+        <is>
+          <t>Grammatica</t>
         </is>
       </c>
       <c r="E27" s="49" t="inlineStr">
@@ -10323,12 +10323,12 @@
       </c>
       <c r="F27" s="56" t="inlineStr">
         <is>
-          <t>Scenario utile ma meno frequente del bar: può slittare alla Fase 2.</t>
+          <t>In/on/at: l'area con più interferenza dall'italiano, serve dall'inizio.</t>
         </is>
       </c>
       <c r="G27" s="56" t="inlineStr">
         <is>
-          <t>COM-A1-002, VOC-A1-001</t>
+          <t>GRA-A1-015</t>
         </is>
       </c>
       <c r="H27" s="46" t="n">
@@ -10341,17 +10341,17 @@
       </c>
       <c r="B28" s="46" t="inlineStr">
         <is>
-          <t>GRA-A1-017</t>
+          <t>COM-A1-003</t>
         </is>
       </c>
       <c r="C28" s="56" t="inlineStr">
         <is>
-          <t>Present continuous: azioni in corso</t>
-        </is>
-      </c>
-      <c r="D28" s="47" t="inlineStr">
-        <is>
-          <t>Grammatica</t>
+          <t>In hotel: fare il check-in</t>
+        </is>
+      </c>
+      <c r="D28" s="51" t="inlineStr">
+        <is>
+          <t>Comunicazione</t>
         </is>
       </c>
       <c r="E28" s="49" t="inlineStr">
@@ -10361,16 +10361,16 @@
       </c>
       <c r="F28" s="56" t="inlineStr">
         <is>
-          <t>Il present continuous manca nella bozza originale ed è irrinunciabile in A1.</t>
+          <t>Scenario utile ma meno frequente del bar: può slittare alla Fase 2.</t>
         </is>
       </c>
       <c r="G28" s="56" t="inlineStr">
         <is>
-          <t>GRA-A1-016</t>
+          <t>COM-A1-002, VOC-A1-001</t>
         </is>
       </c>
       <c r="H28" s="46" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="40">
@@ -10379,12 +10379,12 @@
       </c>
       <c r="B29" s="46" t="inlineStr">
         <is>
-          <t>GRA-A1-018</t>
+          <t>GRA-A1-017</t>
         </is>
       </c>
       <c r="C29" s="56" t="inlineStr">
         <is>
-          <t>Present simple o present continuous?</t>
+          <t>Present continuous: azioni in corso</t>
         </is>
       </c>
       <c r="D29" s="47" t="inlineStr">
@@ -10399,16 +10399,16 @@
       </c>
       <c r="F29" s="56" t="inlineStr">
         <is>
-          <t>Il contrasto simple/continuous previene l'errore più persistente del livello.</t>
+          <t>Il present continuous manca nella bozza originale ed è irrinunciabile in A1.</t>
         </is>
       </c>
       <c r="G29" s="56" t="inlineStr">
         <is>
-          <t>GRA-A1-017, GRA-A1-011</t>
+          <t>GRA-A1-016</t>
         </is>
       </c>
       <c r="H29" s="46" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="30" ht="23.25" customHeight="1" s="40">
@@ -10417,17 +10417,17 @@
       </c>
       <c r="B30" s="46" t="inlineStr">
         <is>
-          <t>COM-A1-005</t>
+          <t>GRA-A1-018</t>
         </is>
       </c>
       <c r="C30" s="56" t="inlineStr">
         <is>
-          <t>Descrivere la propria routine quotidiana</t>
-        </is>
-      </c>
-      <c r="D30" s="51" t="inlineStr">
-        <is>
-          <t>Comunicazione</t>
+          <t>Present simple o present continuous?</t>
+        </is>
+      </c>
+      <c r="D30" s="47" t="inlineStr">
+        <is>
+          <t>Grammatica</t>
         </is>
       </c>
       <c r="E30" s="49" t="inlineStr">
@@ -10437,12 +10437,12 @@
       </c>
       <c r="F30" s="56" t="inlineStr">
         <is>
-          <t>Applica present simple e avverbi in un compito reale.</t>
+          <t>Il contrasto simple/continuous previene l'errore più persistente del livello.</t>
         </is>
       </c>
       <c r="G30" s="56" t="inlineStr">
         <is>
-          <t>COM-A1-003, GRA-A1-011, GRA-A1-013</t>
+          <t>GRA-A1-017, GRA-A1-011</t>
         </is>
       </c>
       <c r="H30" s="46" t="n">
@@ -10455,17 +10455,17 @@
       </c>
       <c r="B31" s="46" t="inlineStr">
         <is>
-          <t>VOC-A1-005</t>
+          <t>COM-A1-005</t>
         </is>
       </c>
       <c r="C31" s="56" t="inlineStr">
         <is>
-          <t>Falsi amici essenziali</t>
-        </is>
-      </c>
-      <c r="D31" s="54" t="inlineStr">
-        <is>
-          <t>Vocabolario</t>
+          <t>Descrivere la propria routine quotidiana</t>
+        </is>
+      </c>
+      <c r="D31" s="51" t="inlineStr">
+        <is>
+          <t>Comunicazione</t>
         </is>
       </c>
       <c r="E31" s="49" t="inlineStr">
@@ -10475,16 +10475,16 @@
       </c>
       <c r="F31" s="56" t="inlineStr">
         <is>
-          <t>I falsi amici sono il tratto distintivo di una app pensata per italiani.</t>
+          <t>Applica present simple e avverbi in un compito reale.</t>
         </is>
       </c>
       <c r="G31" s="56" t="inlineStr">
         <is>
-          <t>VOC-A1-004</t>
+          <t>COM-A1-003, GRA-A1-011, GRA-A1-013</t>
         </is>
       </c>
       <c r="H31" s="46" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="32" ht="23.25" customHeight="1" s="40">
@@ -10493,69 +10493,107 @@
       </c>
       <c r="B32" s="46" t="inlineStr">
         <is>
-          <t>GRA-A2-001</t>
+          <t>VOC-A1-005</t>
         </is>
       </c>
       <c r="C32" s="56" t="inlineStr">
         <is>
-          <t>Past simple del verbo to be</t>
-        </is>
-      </c>
-      <c r="D32" s="47" t="inlineStr">
-        <is>
-          <t>Grammatica</t>
-        </is>
-      </c>
-      <c r="E32" s="58" t="inlineStr">
-        <is>
-          <t>A2</t>
+          <t>Falsi amici essenziali</t>
+        </is>
+      </c>
+      <c r="D32" s="54" t="inlineStr">
+        <is>
+          <t>Vocabolario</t>
+        </is>
+      </c>
+      <c r="E32" s="49" t="inlineStr">
+        <is>
+          <t>A1</t>
         </is>
       </c>
       <c r="F32" s="56" t="inlineStr">
         <is>
-          <t>Primo passo verso l'A2: incluso solo se l'MVP vuole mostrare la progressione.</t>
+          <t>I falsi amici sono il tratto distintivo di una app pensata per italiani.</t>
         </is>
       </c>
       <c r="G32" s="56" t="inlineStr">
         <is>
-          <t>GRA-A1-018</t>
+          <t>VOC-A1-004</t>
         </is>
       </c>
       <c r="H32" s="46" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="33" ht="27.75" customHeight="1" s="40"/>
-    <row r="34" ht="15" customHeight="1" s="40">
-      <c r="B34" s="67" t="inlineStr">
-        <is>
-          <t>Totale lezioni MVP</t>
-        </is>
-      </c>
-      <c r="C34" s="68">
-        <f>COUNTA(B5:B32)</f>
-        <v/>
-      </c>
-    </row>
+    <row r="33" ht="27.75" customHeight="1" s="40">
+      <c r="A33" s="46" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="46" t="inlineStr">
+        <is>
+          <t>GRA-A2-001</t>
+        </is>
+      </c>
+      <c r="C33" s="56" t="inlineStr">
+        <is>
+          <t>Past simple del verbo to be</t>
+        </is>
+      </c>
+      <c r="D33" s="47" t="inlineStr">
+        <is>
+          <t>Grammatica</t>
+        </is>
+      </c>
+      <c r="E33" s="58" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="F33" s="56" t="inlineStr">
+        <is>
+          <t>Primo passo verso l'A2: incluso solo se l'MVP vuole mostrare la progressione.</t>
+        </is>
+      </c>
+      <c r="G33" s="56" t="inlineStr">
+        <is>
+          <t>GRA-A1-018</t>
+        </is>
+      </c>
+      <c r="H33" s="46" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1" s="40"/>
     <row r="35" ht="15" customHeight="1" s="40">
       <c r="B35" s="67" t="inlineStr">
         <is>
-          <t>Durata totale (min)</t>
+          <t>Totale lezioni MVP</t>
         </is>
       </c>
       <c r="C35" s="68">
-        <f>SUM(I5:I32)</f>
+        <f>COUNTA(B5:B33)</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="40">
       <c r="B36" s="67" t="inlineStr">
         <is>
+          <t>Durata totale (min)</t>
+        </is>
+      </c>
+      <c r="C36" s="68">
+        <f>SUM(I5:I33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="67" t="inlineStr">
+        <is>
           <t>Essenziali</t>
         </is>
       </c>
-      <c r="C36" s="68">
-        <f>COUNTIF(F5:F32,"Essenziale")</f>
+      <c r="C37" s="68">
+        <f>COUNTIF(F5:F33,"Essenziale")</f>
         <v/>
       </c>
     </row>

</xml_diff>